<commit_message>
EPBDS-16845 Fix ==== comparing a Float by reference and a float by its digits
Float f = 4.3f; f ==== 4.3 was false and float f = 4.3f; f ==== 4.3 was true.
A strict comparison now takes a float by its binary value, as Java does,
converts mixed numbers to one type, treats NaN and -0.0 as IEEE does for
boxed values too, and supports <==, >==, <=== and >=== for BigDecimal.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Operators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Operators.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N75"/>
+  <dimension ref="B2:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1987,10 +1987,11 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1">
-      <c r="B4" s="2">
-        <f>= and != (or &lt;&gt;) test equality, &lt; &gt; &lt;= &gt;= compare numbers, dates and texts. For fractions == and the other operators ignore the tiny error of binary rounding, so 0.1 + 0.2 == 0.3 is true. The strict operators ==== !=== &lt;== &gt;== &lt;=== &gt;=== compare exactly.</f>
-        <v/>
+    <row r="4" ht="30" customHeight="1">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Operators == and != (or &lt;&gt;) test equality, &lt; &gt; &lt;= &gt;= compare numbers, dates and texts. For fractions == and the other operators ignore the tiny error of binary rounding, so 0.1 + 0.2 == 0.3 is true. The strict operators ==== !=== &lt;== &gt;== &lt;=== &gt;=== compare exactly, and they take a Float by its binary value, as Java does: 4.3f is 4.300000190734863, so 4.3f ==== 4.3 is false.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2516,795 +2517,851 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>FloatStrict</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>= 4.3f ==== 4.3</t>
+        </is>
+      </c>
+    </row>
     <row r="35">
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>FloatBinaryValue</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>= 4.3f ==== 4.300000190734863</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Test RoundingTolerance RoundingToleranceTest</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n"/>
-      <c r="D35" s="8" t="n"/>
-      <c r="E35" s="8" t="n"/>
-      <c r="F35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="9" t="inlineStr">
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>_res_.$Tolerant</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>_res_.$Strict</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>_res_.$StrictNot</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>_res_.$TolerantGreater</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>_res_.$StrictGreater</t>
         </is>
       </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatStrict</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatBinaryValue</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>0.1 + 0.2 == 0.3</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="C39" s="11" t="inlineStr">
         <is>
           <t>====</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D39" s="9" t="inlineStr">
         <is>
           <t>!===</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>&gt;</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>&gt;==</t>
         </is>
       </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="B40" s="2" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>4.3f ==== 4.3</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
+        <is>
+          <t>4.3f ==== 4.300000190734863</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Texts are compared character by character, so "Item10" &lt; "Item9". The operators string== string!= (or string&lt;&gt;) string&lt; string&gt; string&lt;= string&gt;= compare the numbers inside texts as numbers, so "Item10" string&gt; "Item9". For these operators an empty text is less than any other text, while "&lt;" with an empty text gives an empty result.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" s="3" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult TextComparison(String left, String right)</t>
         </is>
       </c>
-      <c r="C42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="B43" s="5" t="inlineStr">
+      <c r="C44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Less</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>= left &lt; right</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>NaturalLess</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>= left string&lt; right</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>NaturalLessOrEqual</t>
+          <t>Less</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>= left string&lt;= right</t>
+          <t>= left &lt; right</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>NaturalGreater</t>
+          <t>NaturalLess</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>= left string&gt; right</t>
+          <t>= left string&lt; right</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>NaturalGreaterOrEqual</t>
+          <t>NaturalLessOrEqual</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>= left string&gt;= right</t>
+          <t>= left string&lt;= right</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>NaturalEqual</t>
+          <t>NaturalGreater</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>= left string== right</t>
+          <t>= left string&gt; right</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>NaturalNotEqual</t>
+          <t>NaturalGreaterOrEqual</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>= left string!= right</t>
+          <t>= left string&gt;= right</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="6" t="inlineStr">
         <is>
+          <t>NaturalEqual</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>= left string== right</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>NaturalNotEqual</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>= left string!= right</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="6" t="inlineStr">
+        <is>
           <t>NaturalNotEqualAlt</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>= left string&lt;&gt; right</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="3" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>Test TextComparison TextComparisonTest</t>
         </is>
       </c>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="8" t="n"/>
-      <c r="E53" s="8" t="n"/>
-      <c r="F53" s="8" t="n"/>
-      <c r="G53" s="8" t="n"/>
-      <c r="H53" s="8" t="n"/>
-      <c r="I53" s="8" t="n"/>
-      <c r="J53" s="8" t="n"/>
-      <c r="K53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="9" t="inlineStr">
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="9" t="inlineStr">
         <is>
           <t>left</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>right</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr">
+      <c r="D56" s="9" t="inlineStr">
         <is>
           <t>_res_.$Less</t>
         </is>
       </c>
-      <c r="E54" s="9" t="inlineStr">
+      <c r="E56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalLess</t>
         </is>
       </c>
-      <c r="F54" s="9" t="inlineStr">
+      <c r="F56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalLessOrEqual</t>
         </is>
       </c>
-      <c r="G54" s="9" t="inlineStr">
+      <c r="G56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalGreater</t>
         </is>
       </c>
-      <c r="H54" s="9" t="inlineStr">
+      <c r="H56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalGreaterOrEqual</t>
         </is>
       </c>
-      <c r="I54" s="9" t="inlineStr">
+      <c r="I56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalEqual</t>
         </is>
       </c>
-      <c r="J54" s="9" t="inlineStr">
+      <c r="J56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalNotEqual</t>
         </is>
       </c>
-      <c r="K54" s="9" t="inlineStr">
+      <c r="K56" s="9" t="inlineStr">
         <is>
           <t>_res_.$NaturalNotEqualAlt</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="5" t="inlineStr">
+    <row r="57">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Left</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Right</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>&lt;</t>
         </is>
       </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>string&lt;</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>string&lt;=</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>string&gt;</t>
         </is>
       </c>
-      <c r="H55" s="5" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>string&gt;=</t>
         </is>
       </c>
-      <c r="I55" s="5" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
         <is>
           <t>string==</t>
         </is>
       </c>
-      <c r="J55" s="5" t="inlineStr">
+      <c r="J57" s="5" t="inlineStr">
         <is>
           <t>string!=</t>
         </is>
       </c>
-      <c r="K55" s="5" t="inlineStr">
+      <c r="K57" s="5" t="inlineStr">
         <is>
           <t>string&lt;&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>Item10</t>
-        </is>
-      </c>
-      <c r="C56" s="6" t="inlineStr">
-        <is>
-          <t>Item9</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E56" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I56" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E57" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F57" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G57" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H57" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I57" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="J57" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="K57" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="6" t="inlineStr">
         <is>
+          <t>Item10</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Item9</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F58" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I58" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J58" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K58" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E59" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F59" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G59" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H59" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I59" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J59" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K59" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="6" t="inlineStr">
+        <is>
           <t>abc</t>
         </is>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C60" s="6" t="inlineStr">
         <is>
           <t>abd</t>
         </is>
       </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G58" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H58" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I58" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E60" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F60" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H60" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I60" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J60" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K60" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="6" t="inlineStr">
         <is>
           <t>abc</t>
         </is>
       </c>
-      <c r="D59" s="10" t="n"/>
-      <c r="E59" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F59" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G59" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H59" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I59" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J59" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K59" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="6" t="n"/>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E60" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F60" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G60" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H60" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I60" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="J60" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="K60" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="16.5" customHeight="1">
-      <c r="B62" s="2" t="inlineStr">
+      <c r="D61" s="10" t="n"/>
+      <c r="E61" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F61" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H61" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I61" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J61" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K61" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E62" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H62" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I62" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J62" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K62" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16.5" customHeight="1">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Dates compare by time, and arrays are equal when all their elements are equal.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="B64" s="3" t="inlineStr">
+    <row r="66">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult DateAndArrayComparison(Date first, Date second)</t>
         </is>
       </c>
-      <c r="C64" s="4" t="n"/>
-    </row>
-    <row r="65">
-      <c r="B65" s="5" t="inlineStr">
+      <c r="C66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>Earlier</t>
-        </is>
-      </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>= first &lt; second</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>SameDay</t>
-        </is>
-      </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>= first == second</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>SameArrays</t>
+          <t>Earlier</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>= new Integer[] {1, 2} == new Integer[] {1, 2}</t>
+          <t>= first &lt; second</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="6" t="inlineStr">
         <is>
+          <t>SameDay</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>= first == second</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>SameArrays</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>= new Integer[] {1, 2} == new Integer[] {1, 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="6" t="inlineStr">
+        <is>
           <t>DifferentArrays</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>= new Integer[] {1, 2} != new Integer[] {2, 1}</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="B71" s="3" t="inlineStr">
+    <row r="73">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>Test DateAndArrayComparison DateAndArrayComparisonTest</t>
         </is>
       </c>
-      <c r="C71" s="8" t="n"/>
-      <c r="D71" s="8" t="n"/>
-      <c r="E71" s="8" t="n"/>
-      <c r="F71" s="8" t="n"/>
-      <c r="G71" s="4" t="n"/>
-    </row>
-    <row r="72">
-      <c r="B72" s="9" t="inlineStr">
+      <c r="C73" s="8" t="n"/>
+      <c r="D73" s="8" t="n"/>
+      <c r="E73" s="8" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="9" t="inlineStr">
         <is>
           <t>first</t>
         </is>
       </c>
-      <c r="C72" s="9" t="inlineStr">
+      <c r="C74" s="9" t="inlineStr">
         <is>
           <t>second</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr">
+      <c r="D74" s="9" t="inlineStr">
         <is>
           <t>_res_.$Earlier</t>
         </is>
       </c>
-      <c r="E72" s="9" t="inlineStr">
+      <c r="E74" s="9" t="inlineStr">
         <is>
           <t>_res_.$SameDay</t>
         </is>
       </c>
-      <c r="F72" s="9" t="inlineStr">
+      <c r="F74" s="9" t="inlineStr">
         <is>
           <t>_res_.$SameArrays</t>
         </is>
       </c>
-      <c r="G72" s="9" t="inlineStr">
+      <c r="G74" s="9" t="inlineStr">
         <is>
           <t>_res_.$DifferentArrays</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" s="5" t="inlineStr">
+    <row r="75">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>First</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>Second</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>Earlier</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr">
         <is>
           <t>Same Day</t>
         </is>
       </c>
-      <c r="F73" s="5" t="inlineStr">
+      <c r="F75" s="5" t="inlineStr">
         <is>
           <t>Same Arrays</t>
         </is>
       </c>
-      <c r="G73" s="5" t="inlineStr">
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>Different Arrays</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="B74" s="6" t="inlineStr">
+    <row r="76">
+      <c r="B76" s="6" t="inlineStr">
         <is>
           <t>2024-01-15</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C76" s="6" t="inlineStr">
         <is>
           <t>2024-03-01</t>
         </is>
       </c>
-      <c r="D74" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E74" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F74" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G74" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" s="6" t="inlineStr">
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E76" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F76" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="6" t="inlineStr">
         <is>
           <t>2024-03-01</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C77" s="6" t="inlineStr">
         <is>
           <t>2024-03-01</t>
         </is>
       </c>
-      <c r="D75" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E75" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F75" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G75" s="10" t="inlineStr">
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G77" s="10" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -3313,16 +3370,16 @@
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B62:I62"/>
-    <mergeCell ref="B40:I40"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B53:K53"/>
-    <mergeCell ref="B71:G71"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B42:I42"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="B55:K55"/>
+    <mergeCell ref="B73:G73"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="B20:N20"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B37:H37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3959,7 +4016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K136"/>
+  <dimension ref="B2:K144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -3982,10 +4039,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1">
+    <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Numbers of different types compare by their values: an Integer equals a Double, a Long or a BigDecimal with the same value. A Float is compared with the tolerance of binary rounding, so it equals the Double written the same way.</t>
+          <t>Numbers of different types compare by their values: an Integer equals a Double, a Long or a BigDecimal with the same value. A Float becomes the Double with the same digits, so 4.3f == 4.3 is true. The strict operators take a Float by its binary value, as Java does, so a Float 4.3f is not strictly equal to a Double 4.3, while a Double is compared with a BigDecimal by its digits.</t>
         </is>
       </c>
     </row>
@@ -4117,92 +4174,72 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>FloatAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>= Float f = 4.3f; Double d = 4.3; f ==== d</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>FloatAndPrimitiveFloatStrict</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>= Float f = 4.3f; float g = 4.3f; f ==== g</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>ExactFloatAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>= float f = 0.5f; f ==== 0.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>DecimalAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>= new BigDecimal("4.3") ==== 4.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Test MixedNumberComparison MixedNumberComparisonTest</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$IntegerAndDouble</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>1 == 1.0</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$IntegerAndFraction</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>1 &gt; -2.5</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$LongAndDecimal</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>5L == new BigDecimal("5.0")</t>
-        </is>
-      </c>
-      <c r="D21" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$LongMoreThanDecimal</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>5L &gt; new BigDecimal("4.5")</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ByteAndBigInteger</t>
+          <t>_res_.$IntegerAndDouble</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>(byte) 7 == new BigInteger("7")</t>
+          <t>1 == 1.0</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -4214,12 +4251,12 @@
     <row r="24">
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ShortAndLong</t>
+          <t>_res_.$IntegerAndFraction</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>(Short) 3 &gt;= 3L</t>
+          <t>1 &gt; -2.5</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
@@ -4231,12 +4268,12 @@
     <row r="25">
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatAndDouble</t>
+          <t>_res_.$LongAndDecimal</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>4.3f == 4.3</t>
+          <t>5L == new BigDecimal("5.0")</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
@@ -4248,489 +4285,493 @@
     <row r="26">
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroAndEmpty</t>
+          <t>_res_.$LongMoreThanDecimal</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Integer a = 0; Double d = null; a == d</t>
+          <t>5L &gt; new BigDecimal("4.5")</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="9" t="inlineStr">
         <is>
+          <t>_res_.$ByteAndBigInteger</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>(byte) 7 == new BigInteger("7")</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ShortAndLong</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>(Short) 3 &gt;= 3L</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatAndDouble</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>4.3f == 4.3</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ZeroAndEmpty</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Integer a = 0; Double d = null; a == d</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
           <t>_res_.$EmptyIntegerAndEmptyDouble</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Integer a = null; Double d = null; a == d</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="B29" s="2" t="inlineStr">
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Float f = 4.3f; Double d = 4.3; f ==== d</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FloatAndPrimitiveFloatStrict</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Float f = 4.3f; float g = 4.3f; f ==== g</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ExactFloatAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>float f = 0.5f; f ==== 0.5</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$DecimalAndDoubleStrict</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>new BigDecimal("4.3") ==== 4.3</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Booleans, characters, texts and dates are ordered too: false is less than true; characters and texts compare by character codes, so they are case-sensitive, capital letters come before small ones and "2" &gt; "10". An empty text "" is not empty (null). Dates compare by time, so a date equals the same date at 00:00.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult OtherTypeComparison()</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="5" t="inlineStr">
+      <c r="C39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>FalseBeforeTrue</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>= false &lt; true</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>EmptyBoolean</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>= Boolean flag = null; flag == false</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>EmptyBooleanOrder</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>= Boolean flag = null; flag &gt; true</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>LetterOrder</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>= 'a' &lt; 'b'</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>CapitalFirst</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>= 'A' &lt; 'a'</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>LetterCase</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>= 'a' == 'A'</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>DigitCharacters</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>= '2' &gt; '1'</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="B40" s="6" t="inlineStr">
-        <is>
-          <t>EmptyCharacter</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>= Character c = null; c &lt; 'B'</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>TextCase</t>
+          <t>FalseBeforeTrue</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>= "Test" == "test"</t>
+          <t>= false &lt; true</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>TextCapitalFirst</t>
+          <t>EmptyBoolean</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>= "Test" &lt; "test"</t>
+          <t>= Boolean flag = null; flag == false</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>TextDigits</t>
+          <t>EmptyBooleanOrder</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>= "2" &gt; "10"</t>
+          <t>= Boolean flag = null; flag &gt; true</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>TextPrefix</t>
+          <t>LetterOrder</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>= "test" &lt; "test1"</t>
+          <t>= 'a' &lt; 'b'</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>EmptyTextIsNotNull</t>
+          <t>CapitalFirst</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>= "" == null</t>
+          <t>= 'A' &lt; 'a'</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>EmptyTextFirst</t>
+          <t>LetterCase</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>= "" &lt; "a"</t>
+          <t>= 'a' == 'A'</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>FarDates</t>
+          <t>DigitCharacters</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>= Date(2000, 10, 13) &lt; Date(3000, 10, 13)</t>
+          <t>= '2' &gt; '1'</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>DateAtMidnight</t>
+          <t>EmptyCharacter</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>= Date(2017, 10, 13) == Date(2017, 10, 13, 0, 0)</t>
+          <t>= Character c = null; c &lt; 'B'</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>DateMinuteLater</t>
+          <t>TextCase</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>= Date(2017, 10, 13) &lt; Date(2017, 10, 13, 0, 1)</t>
+          <t>= "Test" == "test"</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>EmptyDate</t>
+          <t>TextCapitalFirst</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>= Date day = null; day &lt; Date(2017, 10, 13)</t>
+          <t>= "Test" &lt; "test"</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="6" t="inlineStr">
         <is>
+          <t>TextDigits</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>= "2" &gt; "10"</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>TextPrefix</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>= "test" &lt; "test1"</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>EmptyTextIsNotNull</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>= "" == null</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>EmptyTextFirst</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>= "" &lt; "a"</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>FarDates</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>= Date(2000, 10, 13) &lt; Date(3000, 10, 13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>DateAtMidnight</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>= Date(2017, 10, 13) == Date(2017, 10, 13, 0, 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>DateMinuteLater</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>= Date(2017, 10, 13) &lt; Date(2017, 10, 13, 0, 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>EmptyDate</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>= Date day = null; day &lt; Date(2017, 10, 13)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
           <t>TwoEmptyDates</t>
         </is>
       </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr">
         <is>
           <t>= Date day = null; Date other = null; day &gt;= other</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="3" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>Test OtherTypeComparison OtherTypeComparisonTest</t>
         </is>
       </c>
-      <c r="C53" s="8" t="n"/>
-      <c r="D53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$FalseBeforeTrue</t>
-        </is>
-      </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>false &lt; true</t>
-        </is>
-      </c>
-      <c r="D54" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$EmptyBoolean</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Boolean flag = null; flag == false</t>
-        </is>
-      </c>
-      <c r="D55" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$EmptyBooleanOrder</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Boolean flag = null; flag &gt; true</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="n"/>
-    </row>
-    <row r="57">
-      <c r="B57" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$LetterOrder</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>'a' &lt; 'b'</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$CapitalFirst</t>
-        </is>
-      </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>'A' &lt; 'a'</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="B59" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$LetterCase</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>'a' == 'A'</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$DigitCharacters</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>'2' &gt; '1'</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="B61" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$EmptyCharacter</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Character c = null; c &lt; 'B'</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="n"/>
+      <c r="C61" s="8" t="n"/>
+      <c r="D61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TextCase</t>
+          <t>_res_.$FalseBeforeTrue</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>"Test" == "test"</t>
+          <t>false &lt; true</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TextCapitalFirst</t>
+          <t>_res_.$EmptyBoolean</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>"Test" &lt; "test"</t>
+          <t>Boolean flag = null; flag == false</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TextDigits</t>
+          <t>_res_.$EmptyBooleanOrder</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>"2" &gt; "10"</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Boolean flag = null; flag &gt; true</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="n"/>
     </row>
     <row r="65">
       <c r="B65" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TextPrefix</t>
+          <t>_res_.$LetterOrder</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>"test" &lt; "test1"</t>
+          <t>'a' &lt; 'b'</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
@@ -4742,46 +4783,46 @@
     <row r="66">
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyTextIsNotNull</t>
+          <t>_res_.$CapitalFirst</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>"" == null</t>
+          <t>'A' &lt; 'a'</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyTextFirst</t>
+          <t>_res_.$LetterCase</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>"" &lt; "a"</t>
+          <t>'a' == 'A'</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FarDates</t>
+          <t>_res_.$DigitCharacters</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Date(2000, 10, 13) &lt; Date(3000, 10, 13)</t>
+          <t>'2' &gt; '1'</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -4793,926 +4834,1058 @@
     <row r="69">
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DateAtMidnight</t>
+          <t>_res_.$EmptyCharacter</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Date(2017, 10, 13) == Date(2017, 10, 13, 0, 0)</t>
-        </is>
-      </c>
-      <c r="D69" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>Character c = null; c &lt; 'B'</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>_res_.$DateMinuteLater</t>
+          <t>_res_.$TextCase</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Date(2017, 10, 13) &lt; Date(2017, 10, 13, 0, 1)</t>
+          <t>"Test" == "test"</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="B71" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyDate</t>
+          <t>_res_.$TextCapitalFirst</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Date day = null; day &lt; Date(2017, 10, 13)</t>
-        </is>
-      </c>
-      <c r="D71" s="10" t="n"/>
+          <t>"Test" &lt; "test"</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="B72" s="9" t="inlineStr">
         <is>
+          <t>_res_.$TextDigits</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>"2" &gt; "10"</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$TextPrefix</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>"test" &lt; "test1"</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$EmptyTextIsNotNull</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>"" == null</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$EmptyTextFirst</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>"" &lt; "a"</t>
+        </is>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$FarDates</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Date(2000, 10, 13) &lt; Date(3000, 10, 13)</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$DateAtMidnight</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Date(2017, 10, 13) == Date(2017, 10, 13, 0, 0)</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$DateMinuteLater</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Date(2017, 10, 13) &lt; Date(2017, 10, 13, 0, 1)</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$EmptyDate</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Date day = null; day &lt; Date(2017, 10, 13)</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="9" t="inlineStr">
+        <is>
           <t>_res_.$TwoEmptyDates</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
+      <c r="C80" s="5" t="inlineStr">
         <is>
           <t>Date day = null; Date other = null; day &gt;= other</t>
         </is>
       </c>
-      <c r="D72" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="16.5" customHeight="1">
-      <c r="B74" s="2" t="inlineStr">
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="16.5" customHeight="1">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>Arrays are equal when they have the same length and equal elements in the same order. Two empty arrays are equal, but an empty array is not equal to an absent one (null). Elements of different number types compare by value.</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" s="3" t="inlineStr">
+    <row r="84">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult ArrayComparison(String[] a, String[] b)</t>
         </is>
       </c>
-      <c r="C76" s="4" t="n"/>
-    </row>
-    <row r="77">
-      <c r="B77" s="5" t="inlineStr">
+      <c r="C84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>Equal</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>= a == b</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>NotEqual</t>
-        </is>
-      </c>
-      <c r="C79" s="7" t="inlineStr">
-        <is>
-          <t>= a != b</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>Test ArrayComparison ArrayComparisonTest</t>
-        </is>
-      </c>
-      <c r="C81" s="8" t="n"/>
-      <c r="D81" s="8" t="n"/>
-      <c r="E81" s="4" t="n"/>
-    </row>
-    <row r="82">
-      <c r="B82" s="9" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="C82" s="9" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="D82" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$Equal</t>
-        </is>
-      </c>
-      <c r="E82" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$NotEqual</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="5" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D83" s="12" t="inlineStr">
-        <is>
-          <t>==</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>!=</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E84" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="inlineStr">
-        <is>
-          <t>1, 3, 2</t>
-        </is>
-      </c>
-      <c r="D85" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E85" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>1, 2</t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 3</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E86" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
+          <t>Equal</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>= a == b</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="D87" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E87" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="C88" s="6" t="n"/>
-      <c r="D88" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E88" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
+          <t>NotEqual</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>= a != b</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="6" t="n"/>
-      <c r="C89" s="6" t="n"/>
-      <c r="D89" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E89" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Test ArrayComparison ArrayComparisonTest</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="n"/>
+      <c r="D89" s="8" t="n"/>
+      <c r="E89" s="4" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Equal</t>
+        </is>
+      </c>
+      <c r="E90" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NotEqual</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>Spreadsheet SpreadsheetResult ArrayEdgeCases()</t>
-        </is>
-      </c>
-      <c r="C91" s="4" t="n"/>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D91" s="12" t="inlineStr">
+        <is>
+          <t>==</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>!=</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="B92" s="5" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E92" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>EmptyArrays</t>
-        </is>
-      </c>
-      <c r="C93" s="7" t="inlineStr">
-        <is>
-          <t>= new String[0] == new String[0]</t>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>1, 3, 2</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E93" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>EmptyAndNull</t>
-        </is>
-      </c>
-      <c r="C94" s="7" t="inlineStr">
-        <is>
-          <t>= new String[0] == null</t>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E94" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>NullElement</t>
-        </is>
-      </c>
-      <c r="C95" s="7" t="inlineStr">
-        <is>
-          <t>= new String[] {null} == new String[0]</t>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="B96" s="6" t="inlineStr">
         <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E96" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult ArrayEdgeCases()</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="n"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="5" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>EmptyArrays</t>
+        </is>
+      </c>
+      <c r="C101" s="7" t="inlineStr">
+        <is>
+          <t>= new String[0] == new String[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>EmptyAndNull</t>
+        </is>
+      </c>
+      <c r="C102" s="7" t="inlineStr">
+        <is>
+          <t>= new String[0] == null</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>NullElement</t>
+        </is>
+      </c>
+      <c r="C103" s="7" t="inlineStr">
+        <is>
+          <t>= new String[] {null} == new String[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="6" t="inlineStr">
+        <is>
           <t>NullElements</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C104" s="7" t="inlineStr">
         <is>
           <t>= new Integer[] {1, null} == new Integer[] {1, null}</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="B97" s="6" t="inlineStr">
+    <row r="105">
+      <c r="B105" s="6" t="inlineStr">
         <is>
           <t>MissingElement</t>
         </is>
       </c>
-      <c r="C97" s="7" t="inlineStr">
+      <c r="C105" s="7" t="inlineStr">
         <is>
           <t>= new String[] {"1", null, "3"} == new String[] {"1", "3"}</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="B98" s="6" t="inlineStr">
+    <row r="106">
+      <c r="B106" s="6" t="inlineStr">
         <is>
           <t>IntegersAndDoubles</t>
         </is>
       </c>
-      <c r="C98" s="7" t="inlineStr">
+      <c r="C106" s="7" t="inlineStr">
         <is>
           <t>= new Integer[] {1, 2} == new Double[] {1.0, 2.0}</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="B99" s="6" t="inlineStr">
+    <row r="107">
+      <c r="B107" s="6" t="inlineStr">
         <is>
           <t>IntegersAndLongs</t>
         </is>
       </c>
-      <c r="C99" s="7" t="inlineStr">
+      <c r="C107" s="7" t="inlineStr">
         <is>
           <t>= new Integer[] {1, 2} != new Long[] {1L, 2L}</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="B101" s="3" t="inlineStr">
+    <row r="109">
+      <c r="B109" s="3" t="inlineStr">
         <is>
           <t>Test ArrayEdgeCases ArrayEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C101" s="8" t="n"/>
-      <c r="D101" s="4" t="n"/>
-    </row>
-    <row r="102">
-      <c r="B102" s="9" t="inlineStr">
+      <c r="C109" s="8" t="n"/>
+      <c r="D109" s="4" t="n"/>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
         <is>
           <t>_res_.$EmptyArrays</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>new String[0] == new String[0]</t>
         </is>
       </c>
-      <c r="D102" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="9" t="inlineStr">
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="9" t="inlineStr">
         <is>
           <t>_res_.$EmptyAndNull</t>
         </is>
       </c>
-      <c r="C103" s="5" t="inlineStr">
+      <c r="C111" s="5" t="inlineStr">
         <is>
           <t>new String[0] == null</t>
         </is>
       </c>
-      <c r="D103" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="B104" s="9" t="inlineStr">
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="9" t="inlineStr">
         <is>
           <t>_res_.$NullElement</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>new String[] {null} == new String[0]</t>
         </is>
       </c>
-      <c r="D104" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="B105" s="9" t="inlineStr">
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="9" t="inlineStr">
         <is>
           <t>_res_.$NullElements</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>new Integer[] {1, null} == new Integer[] {1, null}</t>
         </is>
       </c>
-      <c r="D105" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="B106" s="9" t="inlineStr">
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="9" t="inlineStr">
         <is>
           <t>_res_.$MissingElement</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
         <is>
           <t>new String[] {"1", null, "3"} == new String[] {"1", "3"}</t>
         </is>
       </c>
-      <c r="D106" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="B107" s="9" t="inlineStr">
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="9" t="inlineStr">
         <is>
           <t>_res_.$IntegersAndDoubles</t>
         </is>
       </c>
-      <c r="C107" s="5" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>new Integer[] {1, 2} == new Double[] {1.0, 2.0}</t>
         </is>
       </c>
-      <c r="D107" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="B108" s="9" t="inlineStr">
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="9" t="inlineStr">
         <is>
           <t>_res_.$IntegersAndLongs</t>
         </is>
       </c>
-      <c r="C108" s="5" t="inlineStr">
+      <c r="C116" s="5" t="inlineStr">
         <is>
           <t>new Integer[] {1, 2} != new Long[] {1L, 2L}</t>
         </is>
       </c>
-      <c r="D108" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="16.5" customHeight="1">
-      <c r="B110" s="2" t="inlineStr">
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="16.5" customHeight="1">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>A vocabulary type compares like its base type: with values of the base type, with other numbers and with arrays.</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="B112" s="3" t="inlineStr">
+    <row r="120">
+      <c r="B120" s="3" t="inlineStr">
         <is>
           <t>Datatype ShoeSize &lt;Integer&gt;</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="B113" s="6" t="n">
+    <row r="121">
+      <c r="B121" s="6" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="114">
-      <c r="B114" s="6" t="n">
+    <row r="122">
+      <c r="B122" s="6" t="n">
         <v>40</v>
       </c>
     </row>
-    <row r="115">
-      <c r="B115" s="6" t="n">
+    <row r="123">
+      <c r="B123" s="6" t="n">
         <v>42</v>
       </c>
     </row>
-    <row r="117">
-      <c r="B117" s="3" t="inlineStr">
+    <row r="125">
+      <c r="B125" s="3" t="inlineStr">
         <is>
           <t>Datatype Priority &lt;String&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="B122" s="3" t="inlineStr">
-        <is>
-          <t>Spreadsheet SpreadsheetResult VocabularyComparison(ShoeSize size, Integer wanted, Priority priority, String level)</t>
-        </is>
-      </c>
-      <c r="C122" s="4" t="n"/>
-    </row>
-    <row r="123">
-      <c r="B123" s="5" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>SameSize</t>
-        </is>
-      </c>
-      <c r="C124" s="7" t="inlineStr">
-        <is>
-          <t>= size == wanted</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>Smaller</t>
-        </is>
-      </c>
-      <c r="C125" s="7" t="inlineStr">
-        <is>
-          <t>= size &lt; wanted</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>SmallerThanFraction</t>
-        </is>
-      </c>
-      <c r="C126" s="7" t="inlineStr">
-        <is>
-          <t>= size &lt; 40.5</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>SamePriority</t>
-        </is>
-      </c>
-      <c r="C127" s="7" t="inlineStr">
-        <is>
-          <t>= priority == level</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="B128" s="6" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult VocabularyComparison(ShoeSize size, Integer wanted, Priority priority, String level)</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="n"/>
+    </row>
+    <row r="131">
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>SameSize</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t>= size == wanted</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>Smaller</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t>= size &lt; wanted</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>SmallerThanFraction</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t>= size &lt; 40.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>SamePriority</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t>= priority == level</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="B136" s="6" t="inlineStr">
+        <is>
           <t>PriorityBefore</t>
         </is>
       </c>
-      <c r="C128" s="7" t="inlineStr">
+      <c r="C136" s="7" t="inlineStr">
         <is>
           <t>= priority &lt; level</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="B129" s="6" t="inlineStr">
+    <row r="137">
+      <c r="B137" s="6" t="inlineStr">
         <is>
           <t>SameSizes</t>
         </is>
       </c>
-      <c r="C129" s="7" t="inlineStr">
+      <c r="C137" s="7" t="inlineStr">
         <is>
           <t>= new ShoeSize[] {size} == new Integer[] {wanted}</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="B131" s="3" t="inlineStr">
+    <row r="139">
+      <c r="B139" s="3" t="inlineStr">
         <is>
           <t>Test VocabularyComparison VocabularyComparisonTest</t>
         </is>
       </c>
-      <c r="C131" s="8" t="n"/>
-      <c r="D131" s="8" t="n"/>
-      <c r="E131" s="8" t="n"/>
-      <c r="F131" s="8" t="n"/>
-      <c r="G131" s="8" t="n"/>
-      <c r="H131" s="8" t="n"/>
-      <c r="I131" s="8" t="n"/>
-      <c r="J131" s="8" t="n"/>
-      <c r="K131" s="4" t="n"/>
-    </row>
-    <row r="132">
-      <c r="B132" s="9" t="inlineStr">
+      <c r="C139" s="8" t="n"/>
+      <c r="D139" s="8" t="n"/>
+      <c r="E139" s="8" t="n"/>
+      <c r="F139" s="8" t="n"/>
+      <c r="G139" s="8" t="n"/>
+      <c r="H139" s="8" t="n"/>
+      <c r="I139" s="8" t="n"/>
+      <c r="J139" s="8" t="n"/>
+      <c r="K139" s="4" t="n"/>
+    </row>
+    <row r="140">
+      <c r="B140" s="9" t="inlineStr">
         <is>
           <t>size</t>
         </is>
       </c>
-      <c r="C132" s="9" t="inlineStr">
+      <c r="C140" s="9" t="inlineStr">
         <is>
           <t>wanted</t>
         </is>
       </c>
-      <c r="D132" s="9" t="inlineStr">
+      <c r="D140" s="9" t="inlineStr">
         <is>
           <t>priority</t>
         </is>
       </c>
-      <c r="E132" s="9" t="inlineStr">
+      <c r="E140" s="9" t="inlineStr">
         <is>
           <t>level</t>
         </is>
       </c>
-      <c r="F132" s="9" t="inlineStr">
+      <c r="F140" s="9" t="inlineStr">
         <is>
           <t>_res_.$SameSize</t>
         </is>
       </c>
-      <c r="G132" s="9" t="inlineStr">
+      <c r="G140" s="9" t="inlineStr">
         <is>
           <t>_res_.$Smaller</t>
         </is>
       </c>
-      <c r="H132" s="9" t="inlineStr">
+      <c r="H140" s="9" t="inlineStr">
         <is>
           <t>_res_.$SmallerThanFraction</t>
         </is>
       </c>
-      <c r="I132" s="9" t="inlineStr">
+      <c r="I140" s="9" t="inlineStr">
         <is>
           <t>_res_.$SamePriority</t>
         </is>
       </c>
-      <c r="J132" s="9" t="inlineStr">
+      <c r="J140" s="9" t="inlineStr">
         <is>
           <t>_res_.$PriorityBefore</t>
         </is>
       </c>
-      <c r="K132" s="9" t="inlineStr">
+      <c r="K140" s="9" t="inlineStr">
         <is>
           <t>_res_.$SameSizes</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="B133" s="5" t="inlineStr">
+    <row r="141">
+      <c r="B141" s="5" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="C133" s="5" t="inlineStr">
+      <c r="C141" s="5" t="inlineStr">
         <is>
           <t>Wanted</t>
         </is>
       </c>
-      <c r="D133" s="5" t="inlineStr">
+      <c r="D141" s="5" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E133" s="5" t="inlineStr">
+      <c r="E141" s="5" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="F133" s="12" t="inlineStr">
+      <c r="F141" s="12" t="inlineStr">
         <is>
           <t>==</t>
         </is>
       </c>
-      <c r="G133" s="5" t="inlineStr">
+      <c r="G141" s="5" t="inlineStr">
         <is>
           <t>&lt;</t>
         </is>
       </c>
-      <c r="H133" s="5" t="inlineStr">
+      <c r="H141" s="5" t="inlineStr">
         <is>
           <t>&lt; 40.5</t>
         </is>
       </c>
-      <c r="I133" s="5" t="inlineStr">
+      <c r="I141" s="5" t="inlineStr">
         <is>
           <t>Same Priority</t>
         </is>
       </c>
-      <c r="J133" s="5" t="inlineStr">
+      <c r="J141" s="5" t="inlineStr">
         <is>
           <t>&lt;</t>
         </is>
       </c>
-      <c r="K133" s="5" t="inlineStr">
+      <c r="K141" s="5" t="inlineStr">
         <is>
           <t>Arrays</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="B134" s="6" t="n">
+    <row r="142">
+      <c r="B142" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="C134" s="6" t="n">
+      <c r="C142" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="D134" s="6" t="inlineStr">
+      <c r="D142" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E134" s="6" t="inlineStr">
+      <c r="E142" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F134" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G134" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="H134" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I134" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="J134" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="K134" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="B135" s="6" t="n">
+      <c r="F142" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G142" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="H142" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I142" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="J142" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="K142" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="C135" s="6" t="n">
+      <c r="C143" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="D135" s="6" t="inlineStr">
+      <c r="D143" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E135" s="6" t="inlineStr">
+      <c r="E143" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="F135" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G135" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H135" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I135" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J135" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K135" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="B136" s="6" t="n">
+      <c r="F143" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G143" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H143" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I143" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J143" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K143" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="C136" s="6" t="n"/>
-      <c r="D136" s="6" t="inlineStr">
+      <c r="C144" s="6" t="n"/>
+      <c r="D144" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E136" s="6" t="inlineStr">
+      <c r="E144" s="6" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="F136" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G136" s="10" t="n"/>
-      <c r="H136" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I136" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="J136" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="K136" s="10" t="inlineStr">
+      <c r="F144" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G144" s="10" t="n"/>
+      <c r="H144" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I144" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="J144" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="K144" s="10" t="inlineStr">
         <is>
           <t>false</t>
         </is>
@@ -5720,19 +5893,19 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="B82:I82"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B131:K131"/>
-    <mergeCell ref="B101:D101"/>
-    <mergeCell ref="B122:C122"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B81:E81"/>
-    <mergeCell ref="B110:I110"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="B139:K139"/>
+    <mergeCell ref="B109:D109"/>
+    <mergeCell ref="B130:C130"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="B61:D61"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B118:I118"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix the Example-4 operator notes saved as formulas that Excel cannot display
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Operators.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Operators.xlsx
@@ -1988,9 +1988,10 @@
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1">
-      <c r="B4" s="2">
-        <f>= and != (or &lt;&gt;) test equality, &lt; &gt; &lt;= &gt;= compare numbers, dates and texts. For fractions == and the other operators ignore the tiny error of binary rounding, so 0.1 + 0.2 == 0.3 is true. The strict operators ==== !=== &lt;== &gt;== &lt;=== &gt;=== compare exactly.</f>
-        <v/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Operators == and != (or &lt;&gt;) test equality, &lt; &gt; &lt;= &gt;= compare numbers, dates and texts. For fractions == and the other operators ignore the tiny error of binary rounding, so 0.1 + 0.2 == 0.3 is true. The strict operators ==== !=== &lt;== &gt;== &lt;=== &gt;=== compare exactly.</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -6376,9 +6377,10 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="2">
-        <f> assigns a value to a variable or a field, and += -= *= /= update it. A cell can hold several expressions separated by ";": they run in order and the last one gives the value. Use "x += 1" instead of the deprecated "x++".</f>
-        <v/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>The operator = assigns a value to a variable or a field, and += -= *= /= update it. A cell can hold several expressions separated by ";": they run in order and the last one gives the value. Use "x += 1" instead of the deprecated "x++".</t>
+        </is>
       </c>
     </row>
     <row r="6">

</xml_diff>